<commit_message>
Painel para inserção de credenciais adm - Versão 1
</commit_message>
<xml_diff>
--- a/planilha2.xlsx
+++ b/planilha2.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -431,36 +431,588 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>8458747138</t>
+          <t>05789392156</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Não encontrado</t>
+          <t>oliveira.catarina</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>07745631173</t>
+          <t>08126430117</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>kevin.magalhaes</t>
+          <t>igor.oliveira.9</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>00883529190</t>
+          <t>08261038122</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>michel.kuriyama</t>
+          <t>natalia.freitas.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>07182539144</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>julia.egreja</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>06440451162</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>camily.contao</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>08368459192</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>carine.frota</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>05781568140</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>maria.scafuto</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>07828726112</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ramos.eduarda</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>03873058154</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>gustavo.silva.23</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>03450167189</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>maria.jennifer</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>05905886130</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>thaissa.guedes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>04570929125</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>guedes.rafael</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>06194188189</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ana.felix.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>07513902160</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>maria.silva.385</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>05633718119</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ana.araujo.46</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>07714931183</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>maria.baptista.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08567772184</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>thayna.maria</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>07673278103</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>beatriz.oliveira.18</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>06530795324</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>thiago.carvalho.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>71070147141</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>serena.pina</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>06726495196</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>emanuele.gomes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>07139591180</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>talita.santos.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>03813284140</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>isabella.anselmo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>73579092200</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>luizete.cordeiro</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>05721211130</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>barbara.moura.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>05504652197</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>maria.campos.24</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>04554481166</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>luisa.schoffen</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>07220397194</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>lucas.ferreira.13</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>02158158158</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>luisa.araujo</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>01032858141</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>brenda.lacerda</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>05524609157</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ana.rodrigues.45</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>06546177161</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>sophia.delmondez</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>07459954110</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>daniela-jesus.dj</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>05674531110</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>manuela.nepomuceno</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>07563244166</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>maria.fortes.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>05229919124</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ana.falkenberg</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>15350067656</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>luma.cardoso</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>05771769193</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>kethenlin.olegario</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>06319249145</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>joyce-miranda.jm</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>07251774119</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Não encontrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>07699198123</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>thuanne.silva</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>08623691180</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>nicole.soares</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>03423307137</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Não encontrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>06917606162</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Não encontrado</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>08093630112</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>yasmin.galvao</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>07661294117</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>gabrielly.vieira</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>01898704198</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>ana.rech</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>07321296130</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>gabriel.fradique</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>70679469133</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>isabella-ramos.ir</t>
         </is>
       </c>
     </row>

</xml_diff>